<commit_message>
Sync amendements PJL 2632 — 1 changement(s) d'état
</commit_message>
<xml_diff>
--- a/data/export_amendements_ce.xlsx
+++ b/data/export_amendements_ce.xlsx
@@ -689,7 +689,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Export généré le 22/06/2026 à 10:01 UTC — 1026 amendements</t>
+          <t>Export généré le 22/06/2026 à 11:01 UTC — 1026 amendements</t>
         </is>
       </c>
     </row>
@@ -1664,9 +1664,9 @@
           <t>EPR</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Non soutenu</t>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>En traitement</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">

</xml_diff>